<commit_message>
Add 4 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 13
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-products.report.xlsx
+++ b/tools/importer/reports/import-products.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>_reportFile</t>
   </si>
@@ -58,13 +58,31 @@
     <t>products</t>
   </si>
   <si>
-    <t>2026-10-14T20:46:21.504Z</t>
+    <t>2026-10-15T09:24:47.840Z</t>
   </si>
   <si>
     <t>HERSHEY'S Milk Chocolate Candy Bars, 9.3 oz, 6 pack</t>
   </si>
   <si>
     <t>https://www.hersheyland.com/products/hersheys-milk-chocolate-candy-bars-9-3-oz-6-pack.html</t>
+  </si>
+  <si>
+    <t>products/reeses-oreo-milk-chocolate-peanut-butter-cups-1-4-oz.report.json</t>
+  </si>
+  <si>
+    <t>00034000458134</t>
+  </si>
+  <si>
+    <t>products/reeses-oreo-milk-chocolate-peanut-butter-cups-1-4-oz</t>
+  </si>
+  <si>
+    <t>2026-10-15T09:25:41.440Z</t>
+  </si>
+  <si>
+    <t>REESE'S OREO® Milk Chocolate Peanut Butter Cups, 1.4 oz</t>
+  </si>
+  <si>
+    <t>https://www.hersheyland.com/products/reeses-oreo-milk-chocolate-peanut-butter-cups-1-4-oz.html</t>
   </si>
 </sst>
 </file>
@@ -453,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -522,6 +540,35 @@
         <v>17</v>
       </c>
     </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>